<commit_message>
test(calculators): update conversion constants via new shared constants test sheet
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/11-wastewater.xlsx
+++ b/packages/calculators/src/modules/test/11-wastewater.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators-internal/packages/calculators/src/modules/test/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05701E81-48AA-EE4B-93F7-2376216C08ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>

</xml_diff>

<commit_message>
feat(calculators): decimal conversion constants, shared via a constants test workbook (#220)
* feat(calculators): update molecular conversion constants to decimal values

* test(calculators): update conversion constants via new shared constants test sheet
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/11-wastewater.xlsx
+++ b/packages/calculators/src/modules/test/11-wastewater.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators-internal/packages/calculators/src/modules/test/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05701E81-48AA-EE4B-93F7-2376216C08ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>

</xml_diff>